<commit_message>
fix: preserve template styles by mutating values only
</commit_message>
<xml_diff>
--- a/public/templates/invoice-template.xlsx
+++ b/public/templates/invoice-template.xlsx
@@ -65,7 +65,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">          NO.</t>
+    <t>NO.</t>
   </si>
   <si>
     <t>Type and size</t>
@@ -861,7 +861,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -940,13 +940,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="179" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="179" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
@@ -967,9 +967,6 @@
     </xf>
     <xf numFmtId="181" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1023,12 +1020,25 @@
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
     <dxf>
       <numFmt numFmtId="179" formatCode="&quot;￥&quot;#,##0.00_);[Red]\(&quot;￥&quot;#,##0.00\)"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="179" formatCode="&quot;￥&quot;#,##0.00_);[Red]\(&quot;￥&quot;#,##0.00\)"/>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="179" formatCode="&quot;￥&quot;#,##0.00_);[Red]\(&quot;￥&quot;#,##0.00\)"/>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="179" formatCode="&quot;￥&quot;#,##0.00_);[Red]\(&quot;￥&quot;#,##0.00\)"/>
+      <alignment horizontal="center"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleLight1" defaultPivotStyle="PivotStyleLight16"/>
@@ -1384,11 +1394,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InvoiceDetails_2" displayName="InvoiceDetails_2" ref="C16:G33" totalsRowShown="0">
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="C16:G33" etc:filterBottomFollowUsedRange="0"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="          NO."/>
+    <tableColumn id="1" name="NO."/>
     <tableColumn id="2" name="Type and size"/>
     <tableColumn id="3" name="     Quantity"/>
-    <tableColumn id="4" name="Price"/>
-    <tableColumn id="5" name="  Total">
+    <tableColumn id="4" name="Price" dataDxfId="0"/>
+    <tableColumn id="5" name="  Total" dataDxfId="1">
       <calculatedColumnFormula>IF(ISBLANK(InvoiceDetails_2[[#This Row],[     Quantity]]),"",(IFERROR(InvoiceDetails_2[[#This Row],[     Quantity]]*InvoiceDetails_2[[#This Row],[Price]],"")))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1400,11 +1410,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="InvoiceDetails_25" displayName="InvoiceDetails_25" ref="C16:G33" totalsRowShown="0">
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="C16:G33" etc:filterBottomFollowUsedRange="0"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="          NO."/>
+    <tableColumn id="1" name="NO."/>
     <tableColumn id="2" name="Type and size"/>
-    <tableColumn id="3" name="     Quantity"/>
-    <tableColumn id="4" name="Price" dataDxfId="0"/>
-    <tableColumn id="5" name="  Total" dataDxfId="1">
+    <tableColumn id="3" name="     Quantity" dataDxfId="2"/>
+    <tableColumn id="4" name="Price" dataDxfId="3"/>
+    <tableColumn id="5" name="  Total" dataDxfId="4">
       <calculatedColumnFormula>IF(ISBLANK(InvoiceDetails_25[[#This Row],[     Quantity]]),"",(IFERROR(InvoiceDetails_25[[#This Row],[     Quantity]]*InvoiceDetails_25[[#This Row],[Price]],"")))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1808,10 +1818,10 @@
       <c r="E17" s="15">
         <v>1</v>
       </c>
-      <c r="F17" s="40">
+      <c r="F17" s="28">
         <v>62</v>
       </c>
-      <c r="G17" s="40">
+      <c r="G17" s="28">
         <f>E17*F17</f>
         <v>62</v>
       </c>
@@ -1826,10 +1836,10 @@
       <c r="E18" s="15">
         <v>1</v>
       </c>
-      <c r="F18" s="40">
+      <c r="F18" s="28">
         <v>86</v>
       </c>
-      <c r="G18" s="40">
+      <c r="G18" s="28">
         <f t="shared" ref="G18:G31" si="0">E18*F18</f>
         <v>86</v>
       </c>
@@ -1844,10 +1854,10 @@
       <c r="E19" s="15">
         <v>1</v>
       </c>
-      <c r="F19" s="40">
+      <c r="F19" s="28">
         <v>115</v>
       </c>
-      <c r="G19" s="40">
+      <c r="G19" s="28">
         <f t="shared" si="0"/>
         <v>115</v>
       </c>
@@ -1862,10 +1872,10 @@
       <c r="E20" s="15">
         <v>1</v>
       </c>
-      <c r="F20" s="40">
+      <c r="F20" s="28">
         <v>98</v>
       </c>
-      <c r="G20" s="40">
+      <c r="G20" s="28">
         <f t="shared" si="0"/>
         <v>98</v>
       </c>
@@ -1880,10 +1890,10 @@
       <c r="E21" s="15">
         <v>1</v>
       </c>
-      <c r="F21" s="40">
+      <c r="F21" s="28">
         <v>80</v>
       </c>
-      <c r="G21" s="40">
+      <c r="G21" s="28">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
@@ -1898,10 +1908,10 @@
       <c r="E22" s="15">
         <v>1</v>
       </c>
-      <c r="F22" s="40">
+      <c r="F22" s="28">
         <v>78</v>
       </c>
-      <c r="G22" s="40">
+      <c r="G22" s="28">
         <f t="shared" si="0"/>
         <v>78</v>
       </c>
@@ -1916,10 +1926,10 @@
       <c r="E23" s="15">
         <v>1</v>
       </c>
-      <c r="F23" s="40">
+      <c r="F23" s="28">
         <v>82</v>
       </c>
-      <c r="G23" s="40">
+      <c r="G23" s="28">
         <f t="shared" si="0"/>
         <v>82</v>
       </c>
@@ -1934,10 +1944,10 @@
       <c r="E24" s="15">
         <v>1</v>
       </c>
-      <c r="F24" s="40">
+      <c r="F24" s="28">
         <v>65</v>
       </c>
-      <c r="G24" s="40">
+      <c r="G24" s="28">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
@@ -1952,10 +1962,10 @@
       <c r="E25" s="15">
         <v>1</v>
       </c>
-      <c r="F25" s="40">
+      <c r="F25" s="28">
         <v>40</v>
       </c>
-      <c r="G25" s="40">
+      <c r="G25" s="28">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
@@ -1970,10 +1980,10 @@
       <c r="E26" s="15">
         <v>1</v>
       </c>
-      <c r="F26" s="40">
+      <c r="F26" s="28">
         <v>36</v>
       </c>
-      <c r="G26" s="40">
+      <c r="G26" s="28">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
@@ -1988,10 +1998,10 @@
       <c r="E27" s="15">
         <v>1</v>
       </c>
-      <c r="F27" s="40">
+      <c r="F27" s="28">
         <v>40</v>
       </c>
-      <c r="G27" s="40">
+      <c r="G27" s="28">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
@@ -2006,10 +2016,10 @@
       <c r="E28" s="15">
         <v>1</v>
       </c>
-      <c r="F28" s="40">
+      <c r="F28" s="28">
         <v>80</v>
       </c>
-      <c r="G28" s="40">
+      <c r="G28" s="28">
         <f>IF(ISBLANK(InvoiceDetails_2[[#This Row],[     Quantity]]),"",(IFERROR(InvoiceDetails_2[[#This Row],[     Quantity]]*InvoiceDetails_2[[#This Row],[Price]],"")))</f>
         <v>80</v>
       </c>
@@ -2024,10 +2034,10 @@
       <c r="E29" s="15">
         <v>1</v>
       </c>
-      <c r="F29" s="40">
+      <c r="F29" s="28">
         <v>328</v>
       </c>
-      <c r="G29" s="40">
+      <c r="G29" s="28">
         <f>E29*F29</f>
         <v>328</v>
       </c>
@@ -2042,10 +2052,10 @@
       <c r="E30" s="15">
         <v>1</v>
       </c>
-      <c r="F30" s="40">
+      <c r="F30" s="28">
         <v>288</v>
       </c>
-      <c r="G30" s="40">
+      <c r="G30" s="28">
         <f>E30*F30</f>
         <v>288</v>
       </c>
@@ -2060,10 +2070,10 @@
       <c r="E31" s="15">
         <v>1</v>
       </c>
-      <c r="F31" s="40">
+      <c r="F31" s="28">
         <v>60</v>
       </c>
-      <c r="G31" s="40">
+      <c r="G31" s="28">
         <f>E31*F31</f>
         <v>60</v>
       </c>
@@ -2078,10 +2088,10 @@
       <c r="E32" s="15">
         <v>1</v>
       </c>
-      <c r="F32" s="40">
+      <c r="F32" s="28">
         <v>62</v>
       </c>
-      <c r="G32" s="40">
+      <c r="G32" s="28">
         <f>E32*F32</f>
         <v>62</v>
       </c>
@@ -2092,8 +2102,8 @@
       <c r="C33" s="17"/>
       <c r="D33" s="39"/>
       <c r="E33" s="39"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="39" t="str">
+      <c r="F33" s="29"/>
+      <c r="G33" s="29" t="str">
         <f>IF(ISBLANK(InvoiceDetails_2[[#This Row],[     Quantity]]),"",(IFERROR(InvoiceDetails_2[[#This Row],[     Quantity]]*InvoiceDetails_2[[#This Row],[Price]],"")))</f>
         <v/>
       </c>
@@ -2104,10 +2114,10 @@
       <c r="C34" s="18"/>
       <c r="D34" s="18"/>
       <c r="E34" s="4"/>
-      <c r="F34" s="18" t="s">
+      <c r="F34" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="G34" s="32">
+      <c r="G34" s="28">
         <f>IFERROR(SUM(InvoiceDetails_2[  Total]),"0")</f>
         <v>1600</v>
       </c>
@@ -2394,11 +2404,15 @@
         <v>1</v>
       </c>
       <c r="D17" s="13"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="28"/>
+      <c r="E17" s="15">
+        <v>1</v>
+      </c>
+      <c r="F17" s="28">
+        <v>1</v>
+      </c>
       <c r="G17" s="28">
-        <f t="shared" ref="G17:G27" si="0">E17*F17</f>
-        <v>0</v>
+        <f>E17*F17</f>
+        <v>1</v>
       </c>
       <c r="H17" s="4"/>
     </row>
@@ -2411,7 +2425,7 @@
       <c r="E18" s="15"/>
       <c r="F18" s="28"/>
       <c r="G18" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G17:G27" si="0">E18*F18</f>
         <v>0</v>
       </c>
       <c r="H18" s="4"/>
@@ -2628,13 +2642,13 @@
       <c r="B34" s="4"/>
       <c r="C34" s="18"/>
       <c r="D34" s="18"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="30" t="s">
+      <c r="E34" s="30"/>
+      <c r="F34" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="G34" s="31">
+      <c r="G34" s="28">
         <f>IFERROR(SUM(InvoiceDetails_25[  Total]),"0")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34" s="4"/>
     </row>

</xml_diff>